<commit_message>
Added cost and construction_time handle
</commit_message>
<xml_diff>
--- a/Database/260424_MIVES_weights.xlsx
+++ b/Database/260424_MIVES_weights.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanbieg/Documents/Master Thesis/1_Code/Python Repository/SDSD_Bieg/Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{138C38FE-543B-6D4F-8DBE-D05645A7F0E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A3BBD42-D33F-8143-872B-66B956AF1210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3500" yWindow="-17880" windowWidth="24220" windowHeight="15940" xr2:uid="{C87B0895-C1AD-874F-B04F-2F3A4E3CB4D6}"/>
+    <workbookView xWindow="9400" yWindow="-16680" windowWidth="24220" windowHeight="15940" activeTab="1" xr2:uid="{C87B0895-C1AD-874F-B04F-2F3A4E3CB4D6}"/>
   </bookViews>
   <sheets>
     <sheet name="Balanced" sheetId="1" r:id="rId1"/>
+    <sheet name="Input" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="58">
   <si>
     <t>Requirement</t>
   </si>
@@ -99,13 +100,125 @@
   </si>
   <si>
     <t>I5 mtot</t>
+  </si>
+  <si>
+    <t>'241.661.112</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beton für Deckenplatten liefern, einbauen und verdichten. Beton Typ NPK A. Horizontal oder einseitig geneigt bis % 5,0. Plattendicke m 0,21 bis 0,30. </t>
+  </si>
+  <si>
+    <t>NPK Position</t>
+  </si>
+  <si>
+    <t>'364.921.111</t>
+  </si>
+  <si>
+    <t>Beschwerungs- und Schutzschichten. Lose aufbringen. Rundkies gewaschen (Betonkies ungebrochen, gewaschen), Korngruppe 8/16. d mm 50.</t>
+  </si>
+  <si>
+    <t>m2</t>
+  </si>
+  <si>
+    <t>'335.531.114</t>
+  </si>
+  <si>
+    <t>Geschossdecke aus Brettstapeln, Konstruktion, sagerohen Lamellen, h mm 240</t>
+  </si>
+  <si>
+    <t>'661.611.113</t>
+  </si>
+  <si>
+    <t>Zementestriche CT. Beanspruchskategorie A, Festigkeitsklasse C20 - F4, auf Trennschicht. d mm 60</t>
+  </si>
+  <si>
+    <t>'661.433.114</t>
+  </si>
+  <si>
+    <t>Trittschall-Dämmplatten aus expandiertem Polystyrol gewalkt EPS-T. Einlagig mit Randstreifen. Platten unbelegt, d mm 22/20</t>
+  </si>
+  <si>
+    <t>m3</t>
+  </si>
+  <si>
+    <t>'241.511.123</t>
+  </si>
+  <si>
+    <t>Stabstähle. Stahl B500A, liefern und verlegen. BG 1 (1). d mm 16 bis 22.</t>
+  </si>
+  <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>MATERIAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+ready_mixed_concrete</t>
+  </si>
+  <si>
+    <t>Kies gebrochen</t>
+  </si>
+  <si>
+    <t>Steinwolle</t>
+  </si>
+  <si>
+    <t>Unteragsboden Zement, 85 mm</t>
+  </si>
+  <si>
+    <t>steel_reinforcing_bar</t>
+  </si>
+  <si>
+    <t>'241.261.301</t>
+  </si>
+  <si>
+    <t>Schalungen für horizontale Deckenplatten-Untersichten. Typ 3-1 Plattendicke m 0.36 bis 0.45 Spriesshöhe m 3.51 - 5.50. Ohne Ueberhöhung. LE = m2</t>
+  </si>
+  <si>
+    <t>Glue_laminated_timber</t>
+  </si>
+  <si>
+    <t>Ann.</t>
+  </si>
+  <si>
+    <t>Solid_structural_timber</t>
+  </si>
+  <si>
+    <t>prestressing steel</t>
+  </si>
+  <si>
+    <t>wh/m2</t>
+  </si>
+  <si>
+    <t>wh/kg</t>
+  </si>
+  <si>
+    <t>wh/m3</t>
+  </si>
+  <si>
+    <t>logistics, propping, leveling, oiling, cleaning</t>
+  </si>
+  <si>
+    <t>placing</t>
+  </si>
+  <si>
+    <t>placing, stressing</t>
+  </si>
+  <si>
+    <t>placing, vibrating, leveling, cleaning</t>
+  </si>
+  <si>
+    <t>logistics, connections</t>
+  </si>
+  <si>
+    <t>placing, leveling, cleaning</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -117,6 +230,36 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Aptos"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -139,7 +282,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -147,11 +290,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="hair">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFC9C9C9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFC9C9C9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -166,6 +322,22 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -729,4 +901,274 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A3CF732-641D-AF4F-98DB-043B18418DE5}">
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="32.33203125" style="10" customWidth="1"/>
+    <col min="2" max="2" width="32.5" style="10" customWidth="1"/>
+    <col min="3" max="3" width="102.83203125" style="10" customWidth="1"/>
+    <col min="4" max="5" width="27" style="10" customWidth="1"/>
+    <col min="6" max="6" width="34.5" style="10" customWidth="1"/>
+    <col min="7" max="16384" width="10.83203125" style="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A1" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.2">
+      <c r="A2" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="9">
+        <v>75.709999999999994</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" s="10">
+        <v>0.7</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15" x14ac:dyDescent="0.2">
+      <c r="A3" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="9">
+        <v>2.0099999999999998</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" s="10">
+        <f>9/1000</f>
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="10">
+        <v>6</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" s="10">
+        <f>20/1000</f>
+        <v>0.02</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.2">
+      <c r="A5" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="9">
+        <v>205.29</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="10">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="9">
+        <v>1200</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="9">
+        <v>1040</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D8" s="9">
+        <v>12.66</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" s="10">
+        <v>0.2</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="9">
+        <v>6.71</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" s="10">
+        <v>0.2</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="9">
+        <v>23.45</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" s="10">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Worked on plot layout, Vibration for slabs, plastic redistributions in slabs (LL and PL-eingespannt)
</commit_message>
<xml_diff>
--- a/Database/260424_MIVES_weights.xlsx
+++ b/Database/260424_MIVES_weights.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanbieg/Documents/Master Thesis/1_Code/Python Repository/SDSD_Bieg/Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F765FB4-55AE-264E-9BC9-0855FC6C3742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F71D492B-F150-9748-BAA8-55A70FDC6D9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3580" yWindow="960" windowWidth="20800" windowHeight="15940" activeTab="1" xr2:uid="{C87B0895-C1AD-874F-B04F-2F3A4E3CB4D6}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="64">
   <si>
     <t>Requirement</t>
   </si>
@@ -224,13 +224,19 @@
   </si>
   <si>
     <t>Beschreibung</t>
+  </si>
+  <si>
+    <t>'335.531.114</t>
+  </si>
+  <si>
+    <t>Geschossdecke aus Brettstapeln, Konstruktion, sagerohen Lamellen, h mm 240</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -279,6 +285,17 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -325,7 +342,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -357,7 +374,10 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -883,7 +903,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A3CF732-641D-AF4F-98DB-043B18418DE5}">
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32.33203125" style="4" customWidth="1"/>
@@ -898,7 +918,7 @@
     <col min="10" max="16384" width="10.83203125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" ht="15" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>25</v>
       </c>
@@ -926,10 +946,8 @@
       <c r="I1" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-    </row>
-    <row r="2" spans="1:11" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:9" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="8" t="s">
         <v>26</v>
       </c>
@@ -958,7 +976,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" ht="15" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
         <v>27</v>
       </c>
@@ -988,7 +1006,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
         <v>32</v>
       </c>
@@ -1018,7 +1036,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="30" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
         <v>26</v>
       </c>
@@ -1047,7 +1065,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
         <v>30</v>
       </c>
@@ -1058,7 +1076,8 @@
         <v>52</v>
       </c>
       <c r="D6" s="11">
-        <v>2200</v>
+        <f>D7+500</f>
+        <v>1750</v>
       </c>
       <c r="E6" s="12" t="s">
         <v>58</v>
@@ -1076,18 +1095,18 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>52</v>
+      <c r="B7" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>63</v>
       </c>
       <c r="D7" s="11">
-        <v>1700</v>
+        <v>1250</v>
       </c>
       <c r="E7" s="12" t="s">
         <v>58</v>
@@ -1105,12 +1124,12 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>45</v>
       </c>
@@ -1139,7 +1158,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>46</v>
       </c>
@@ -1168,7 +1187,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>47</v>
       </c>
@@ -1197,7 +1216,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>48</v>
       </c>
@@ -1226,7 +1245,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>49</v>
       </c>

</xml_diff>